<commit_message>
Ajout colonne Payé après Dons dans sponsors.xlsx
</commit_message>
<xml_diff>
--- a/sponsors.xlsx
+++ b/sponsors.xlsx
@@ -8,12 +8,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Nom du sponsor</t>
   </si>
   <si>
     <t>Dons</t>
+  </si>
+  <si>
+    <t>Payé</t>
   </si>
   <si>
     <t>Equipements</t>
@@ -106,68 +109,77 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>1000</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2">
         <v>300</v>
       </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
+      <c r="G2" t="s">
+        <v>11</v>
       </c>
       <c r="H2">
-        <f>E2+G2</f>
+        <v>0</v>
       </c>
       <c r="I2">
-        <f>B2-H2</f>
+        <f>F2+H2</f>
+      </c>
+      <c r="J2">
+        <f>B2-I2</f>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3">
         <v>2000</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3">
         <v>500</v>
       </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3">
+      <c r="G3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3">
         <v>200</v>
       </c>
-      <c r="H3">
-        <f>E3+G3</f>
-      </c>
       <c r="I3">
-        <f>B3-H3</f>
+        <f>F3+H3</f>
+      </c>
+      <c r="J3">
+        <f>B3-I3</f>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4">
         <v>1500</v>
@@ -176,56 +188,62 @@
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4">
         <v>150</v>
       </c>
-      <c r="H4">
-        <f>E4+G4</f>
-      </c>
       <c r="I4">
-        <f>B4-H4</f>
+        <f>F4+H4</f>
+      </c>
+      <c r="J4">
+        <f>B4-I4</f>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5">
         <v>3000</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5">
         <v>400</v>
       </c>
-      <c r="F5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
+      <c r="G5" t="s">
+        <v>11</v>
       </c>
       <c r="H5">
-        <f>E5+G5</f>
+        <v>0</v>
       </c>
       <c r="I5">
-        <f>B5-H5</f>
+        <f>F5+H5</f>
+      </c>
+      <c r="J5">
+        <f>B5-I5</f>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <v>800</v>
@@ -234,42 +252,45 @@
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>11</v>
       </c>
       <c r="H6">
-        <f>E6+G6</f>
+        <v>0</v>
       </c>
       <c r="I6">
-        <f>B6-H6</f>
+        <f>F6+H6</f>
+      </c>
+      <c r="J6">
+        <f>B6-I6</f>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <f>SUM(B2:B6)</f>
       </c>
-      <c r="E7">
-        <f>SUM(E2:E6)</f>
-      </c>
-      <c r="G7">
-        <f>SUM(G2:G6)</f>
+      <c r="F7">
+        <f>SUM(F2:F6)</f>
       </c>
       <c r="H7">
         <f>SUM(H2:H6)</f>
       </c>
       <c r="I7">
         <f>SUM(I2:I6)</f>
+      </c>
+      <c r="J7">
+        <f>SUM(J2:J6)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>